<commit_message>
modificacion para trabajar por separado cada seccion e implementacion basica de un menu principal de pendiendo el rango de la institucion
</commit_message>
<xml_diff>
--- a/alumnos/RAC  ENERO MERIDA 2026 ESCUELA JUANA RAMIREZ.xlsx
+++ b/alumnos/RAC  ENERO MERIDA 2026 ESCUELA JUANA RAMIREZ.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Project\alumnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3532051-089C-414D-A694-550BE30B78B4}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BC9DAC-F9F2-43EC-A315-21F95AF00C10}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1063,7 +1063,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd&quot; / &quot;mm&quot; / &quot;yyyy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1075,28 +1075,33 @@
       <sz val="16"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1122,6 +1127,7 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1721,7 +1727,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BG24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
@@ -1776,7 +1782,7 @@
     <col min="59" max="59" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:59" ht="21">
+    <row r="1" spans="1:59" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>329</v>
       </c>
@@ -1839,7 +1845,7 @@
       <c r="BF1" s="4"/>
       <c r="BG1" s="4"/>
     </row>
-    <row r="2" spans="1:59">
+    <row r="2" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1924,7 +1930,7 @@
       <c r="BF2" s="7"/>
       <c r="BG2" s="12"/>
     </row>
-    <row r="3" spans="1:59" ht="100.5" customHeight="1">
+    <row r="3" spans="1:59" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>4</v>
       </c>
@@ -2089,7 +2095,7 @@
       </c>
       <c r="BG3" s="14"/>
     </row>
-    <row r="4" spans="1:59" ht="30">
+    <row r="4" spans="1:59" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>54</v>
       </c>
@@ -2268,7 +2274,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:59" s="20" customFormat="1">
+    <row r="5" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="24">
         <v>17238770</v>
       </c>
@@ -2447,7 +2453,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="6" spans="1:59" s="20" customFormat="1">
+    <row r="6" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="24">
         <v>17129781</v>
       </c>
@@ -2626,7 +2632,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="7" spans="1:59" s="20" customFormat="1">
+    <row r="7" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="24">
         <v>15031556</v>
       </c>
@@ -2805,7 +2811,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="8" spans="1:59" s="20" customFormat="1">
+    <row r="8" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="24">
         <v>22655385</v>
       </c>
@@ -2984,7 +2990,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="9" spans="1:59" s="20" customFormat="1">
+    <row r="9" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="24">
         <v>20850552</v>
       </c>
@@ -3163,7 +3169,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="10" spans="1:59" s="20" customFormat="1">
+    <row r="10" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="24">
         <v>17340678</v>
       </c>
@@ -3342,7 +3348,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="11" spans="1:59" s="20" customFormat="1">
+    <row r="11" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24">
         <v>14700233</v>
       </c>
@@ -3521,7 +3527,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="12" spans="1:59" s="20" customFormat="1">
+    <row r="12" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
         <v>17238934</v>
       </c>
@@ -3700,7 +3706,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="13" spans="1:59" s="20" customFormat="1">
+    <row r="13" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="24">
         <v>18309890</v>
       </c>
@@ -3879,7 +3885,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="14" spans="1:59" s="20" customFormat="1">
+    <row r="14" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24">
         <v>17130801</v>
       </c>
@@ -4058,7 +4064,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="1:59" s="20" customFormat="1">
+    <row r="15" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="24">
         <v>27780603</v>
       </c>
@@ -4237,7 +4243,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="16" spans="1:59" s="20" customFormat="1">
+    <row r="16" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="24">
         <v>24229244</v>
       </c>
@@ -4416,7 +4422,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="17" spans="1:59" s="20" customFormat="1">
+    <row r="17" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="24">
         <v>11951936</v>
       </c>
@@ -4595,7 +4601,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="18" spans="1:59" s="20" customFormat="1">
+    <row r="18" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="35">
         <v>14588010</v>
       </c>
@@ -4774,7 +4780,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="19" spans="1:59" s="20" customFormat="1">
+    <row r="19" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="35">
         <v>12779931</v>
       </c>
@@ -4953,7 +4959,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:59" s="20" customFormat="1">
+    <row r="20" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="35">
         <v>14700020</v>
       </c>
@@ -5132,7 +5138,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="21" spans="1:59" s="20" customFormat="1">
+    <row r="21" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="35">
         <v>17896479</v>
       </c>
@@ -5311,7 +5317,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="22" spans="1:59" s="20" customFormat="1">
+    <row r="22" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="35">
         <v>14588507</v>
       </c>
@@ -5490,7 +5496,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="23" spans="1:59" s="20" customFormat="1">
+    <row r="23" spans="1:59" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="35">
         <v>22655622</v>
       </c>
@@ -5669,7 +5675,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="24" spans="1:59" outlineLevel="1">
+    <row r="24" spans="1:59" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A24" s="44">
         <v>11953316</v>
       </c>

</xml_diff>